<commit_message>
Add database initialization and session management functionality
- Implemented the create_db_and_tables function in app/database.py to set up the database and its tables using SQLModel.
- Added a get_session function in app/database.py to facilitate session management.
- Updated app/dependencies.py to import and utilize the get_session function for dependency injection.
- Ensured that the database engine is created with echo=True for better debugging during development.
</commit_message>
<xml_diff>
--- a/data/embloyees .1.xlsx
+++ b/data/embloyees .1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\خاص احمد جعفر\برمجة\مشاريع\hr_fastapi\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D41F64-7103-4861-A37D-A98F58808210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73131D0F-6039-4DD1-9EA5-DB939C46A3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{74AFE193-51C4-4EE6-8E2A-51EA9F370EF1}"/>
   </bookViews>
@@ -7024,15 +7024,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="19">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -7060,14 +7052,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7280,6 +7264,14 @@
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color auto="1"/>
@@ -7326,23 +7318,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7E524CDE-EFB4-4E89-96B7-A45C6F813777}" name="Table133" displayName="Table133" ref="A1:K2031" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7E524CDE-EFB4-4E89-96B7-A45C6F813777}" name="Table133" displayName="Table133" ref="A1:K2031" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="A1:K2031" xr:uid="{7331ABE9-D21B-4D40-8202-37AD81799F21}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K2031">
-    <sortCondition sortBy="cellColor" ref="C1:C2031" dxfId="4"/>
+    <sortCondition sortBy="cellColor" ref="C1:C2031" dxfId="14"/>
   </sortState>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{3BD77A86-144E-4075-87D9-866CE1D61DAD}" name="Legacy_Code" dataDxfId="15"/>
-    <tableColumn id="90" xr3:uid="{A0B3608E-8905-4736-91D2-C7AD62D17B92}" name="National_ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{453A9229-F3CF-4E9E-8B6C-62120917E40B}" name="Full_Name" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{63669E64-7E60-4F6A-97DD-74819A8C3389}" name="Job_Title" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{63DE3D06-B020-43C8-9929-67296FD45243}" name="Hire_Date" dataDxfId="11"/>
-    <tableColumn id="55" xr3:uid="{0C077F94-E2EC-4087-8022-A30DDF185CE6}" name="Company_Name" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{5FFBEF4E-CA97-4113-93D7-9E60C0449F5D}" name="Site_Name" dataDxfId="9"/>
-    <tableColumn id="65" xr3:uid="{3F1375BF-0752-41D1-8920-3CAF9EB11ED1}" name="Cost_Center" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{83967A1D-19CE-4202-8D7B-9CEA0D2A07D8}" name="Insurance_Status" dataDxfId="7"/>
-    <tableColumn id="91" xr3:uid="{215325F7-C3BA-4B60-9B7F-CCAF60D79359}" name="Employee_Category" dataDxfId="6"/>
-    <tableColumn id="57" xr3:uid="{3C4E6ABC-761D-42E1-9885-1C93194BDC22}" name="Work_Status" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{3BD77A86-144E-4075-87D9-866CE1D61DAD}" name="Legacy_Code" dataDxfId="13"/>
+    <tableColumn id="90" xr3:uid="{A0B3608E-8905-4736-91D2-C7AD62D17B92}" name="National_ID" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{453A9229-F3CF-4E9E-8B6C-62120917E40B}" name="Full_Name" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{63669E64-7E60-4F6A-97DD-74819A8C3389}" name="Job_Title" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{63DE3D06-B020-43C8-9929-67296FD45243}" name="Hire_Date" dataDxfId="9"/>
+    <tableColumn id="55" xr3:uid="{0C077F94-E2EC-4087-8022-A30DDF185CE6}" name="Company_Name" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{5FFBEF4E-CA97-4113-93D7-9E60C0449F5D}" name="Site_Name" dataDxfId="7"/>
+    <tableColumn id="65" xr3:uid="{3F1375BF-0752-41D1-8920-3CAF9EB11ED1}" name="Cost_Center" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{83967A1D-19CE-4202-8D7B-9CEA0D2A07D8}" name="Insurance_Status" dataDxfId="5"/>
+    <tableColumn id="91" xr3:uid="{215325F7-C3BA-4B60-9B7F-CCAF60D79359}" name="Employee_Category" dataDxfId="4"/>
+    <tableColumn id="57" xr3:uid="{3C4E6ABC-761D-42E1-9885-1C93194BDC22}" name="Work_Status" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7653,9 +7645,11 @@
     <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="16" bestFit="1" customWidth="1"/>
@@ -73809,13 +73803,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A32177:A1048576 A1:A2031">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2070:C1048576 C1:C2031">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>